<commit_message>
Parcial update of the values for publishing ov Release 10.0.2
</commit_message>
<xml_diff>
--- a/data/aircraft_operating_costs.xlsx
+++ b/data/aircraft_operating_costs.xlsx
@@ -1,85 +1,68 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oburdash\dev\repos\standard_inputs\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A069D25-09D4-456D-903D-12FDB59B59BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74F48EB9-77F1-45EE-B50C-C60F7E9BE3E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="aircraft_operating_costs" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>B737 NG</t>
   </si>
   <si>
-    <t>33.11 </t>
-  </si>
-  <si>
     <t>A320 Family</t>
   </si>
   <si>
-    <t>36.92 </t>
-  </si>
-  <si>
     <t>B737 Classic</t>
   </si>
   <si>
-    <t>25.28 </t>
-  </si>
-  <si>
     <t>B777</t>
   </si>
   <si>
-    <t>22.07 </t>
-  </si>
-  <si>
     <t>A330</t>
   </si>
   <si>
-    <t>24.48 </t>
-  </si>
-  <si>
     <t>B757</t>
   </si>
   <si>
-    <t>30.51 </t>
-  </si>
-  <si>
     <t>B767</t>
   </si>
   <si>
-    <t>22.18 </t>
-  </si>
-  <si>
     <t>B787</t>
   </si>
   <si>
-    <t>19.86 </t>
-  </si>
-  <si>
     <t>EMB-190</t>
   </si>
   <si>
-    <t>54.00 </t>
-  </si>
-  <si>
     <t>Dash 8</t>
-  </si>
-  <si>
-    <t>58.08 </t>
   </si>
   <si>
     <t>Aircraft.type</t>
@@ -581,8 +564,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -951,225 +935,231 @@
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B1" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C1" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="D1" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="E1" t="s">
-        <v>24</v>
+        <v>14</v>
       </c>
       <c r="F1" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>0</v>
       </c>
-      <c r="B2">
-        <v>14.11</v>
-      </c>
-      <c r="C2">
-        <v>4337</v>
-      </c>
-      <c r="D2">
-        <v>9231</v>
-      </c>
-      <c r="E2">
-        <v>3.76</v>
-      </c>
-      <c r="F2" t="s">
-        <v>1</v>
+      <c r="B2" s="1">
+        <v>15.779920875420876</v>
+      </c>
+      <c r="C2" s="1">
+        <v>4850.2846801346805</v>
+      </c>
+      <c r="D2" s="1">
+        <v>10323.490404040405</v>
+      </c>
+      <c r="E2" s="1">
+        <v>4.2049966329966333</v>
+      </c>
+      <c r="F2" s="1">
+        <v>37.028574074074079</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>12.84</v>
-      </c>
-      <c r="C3">
-        <v>4829</v>
-      </c>
-      <c r="D3">
-        <v>8851</v>
-      </c>
-      <c r="E3">
-        <v>3.6</v>
-      </c>
-      <c r="F3" t="s">
-        <v>3</v>
+        <v>1</v>
+      </c>
+      <c r="B3" s="1">
+        <v>14.359616161616163</v>
+      </c>
+      <c r="C3" s="1">
+        <v>5400.5129629629637</v>
+      </c>
+      <c r="D3" s="1">
+        <v>9898.5173400673411</v>
+      </c>
+      <c r="E3" s="1">
+        <v>4.0260606060606063</v>
+      </c>
+      <c r="F3" s="1">
+        <v>41.28948821548822</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4">
-        <v>8.26</v>
-      </c>
-      <c r="C4">
-        <v>2683</v>
-      </c>
-      <c r="D4">
-        <v>5366</v>
-      </c>
-      <c r="E4">
-        <v>2.96</v>
-      </c>
-      <c r="F4" t="s">
-        <v>5</v>
+        <v>2</v>
+      </c>
+      <c r="B4" s="1">
+        <v>9.2375723905723905</v>
+      </c>
+      <c r="C4" s="1">
+        <v>3000.533501683502</v>
+      </c>
+      <c r="D4" s="1">
+        <v>6001.067003367004</v>
+      </c>
+      <c r="E4" s="1">
+        <v>3.3103164983164985</v>
+      </c>
+      <c r="F4" s="1">
+        <v>28.271892255892258</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B5">
-        <v>40.01</v>
-      </c>
-      <c r="C5">
-        <v>9507</v>
-      </c>
-      <c r="D5">
-        <v>60367</v>
-      </c>
-      <c r="E5">
-        <v>3.53</v>
-      </c>
-      <c r="F5" t="s">
-        <v>7</v>
+        <v>3</v>
+      </c>
+      <c r="B5" s="1">
+        <v>44.745190235690238</v>
+      </c>
+      <c r="C5" s="1">
+        <v>10632.155050505051</v>
+      </c>
+      <c r="D5" s="1">
+        <v>67511.444612794614</v>
+      </c>
+      <c r="E5" s="1">
+        <v>3.9477760942760942</v>
+      </c>
+      <c r="F5" s="1">
+        <v>24.681988215488218</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6">
-        <v>29.87</v>
-      </c>
-      <c r="C6">
-        <v>7827</v>
-      </c>
-      <c r="D6">
-        <v>35857</v>
-      </c>
-      <c r="E6">
-        <v>3.61</v>
-      </c>
-      <c r="F6" t="s">
-        <v>9</v>
+        <v>4</v>
+      </c>
+      <c r="B6" s="1">
+        <v>33.405119528619529</v>
+      </c>
+      <c r="C6" s="1">
+        <v>8753.3267676767682</v>
+      </c>
+      <c r="D6" s="1">
+        <v>40100.681986531992</v>
+      </c>
+      <c r="E6" s="1">
+        <v>4.0372441077441081</v>
+      </c>
+      <c r="F6" s="1">
+        <v>27.377212121212125</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7">
-        <v>18.21</v>
-      </c>
-      <c r="C7">
-        <v>5357</v>
-      </c>
-      <c r="D7">
-        <v>18508</v>
-      </c>
-      <c r="E7">
-        <v>3.73</v>
-      </c>
-      <c r="F7" t="s">
-        <v>11</v>
+        <v>5</v>
+      </c>
+      <c r="B7" s="1">
+        <v>20.365156565656569</v>
+      </c>
+      <c r="C7" s="1">
+        <v>5991.0018518518518</v>
+      </c>
+      <c r="D7" s="1">
+        <v>20698.424915824919</v>
+      </c>
+      <c r="E7" s="1">
+        <v>4.1714461279461279</v>
+      </c>
+      <c r="F7" s="1">
+        <v>34.120863636363637</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8">
-        <v>26</v>
-      </c>
-      <c r="C8">
-        <v>6675</v>
-      </c>
-      <c r="D8">
-        <v>40899</v>
-      </c>
-      <c r="E8">
-        <v>3.61</v>
-      </c>
-      <c r="F8" t="s">
-        <v>13</v>
+        <v>6</v>
+      </c>
+      <c r="B8" s="1">
+        <v>29.07710437710438</v>
+      </c>
+      <c r="C8" s="1">
+        <v>7464.9873737373746</v>
+      </c>
+      <c r="D8" s="1">
+        <v>45739.403535353536</v>
+      </c>
+      <c r="E8" s="1">
+        <v>4.0372441077441081</v>
+      </c>
+      <c r="F8" s="1">
+        <v>24.805006734006735</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>14</v>
-      </c>
-      <c r="B9">
-        <v>30.58</v>
-      </c>
-      <c r="C9">
-        <v>7184</v>
-      </c>
-      <c r="D9">
-        <v>50827</v>
-      </c>
-      <c r="E9">
-        <v>3.11</v>
-      </c>
-      <c r="F9" t="s">
-        <v>15</v>
+        <v>7</v>
+      </c>
+      <c r="B9" s="1">
+        <v>34.199148148148147</v>
+      </c>
+      <c r="C9" s="1">
+        <v>8034.2276094276103</v>
+      </c>
+      <c r="D9" s="1">
+        <v>56842.384006734013</v>
+      </c>
+      <c r="E9" s="1">
+        <v>3.4780690235690237</v>
+      </c>
+      <c r="F9" s="1">
+        <v>22.210434343434343</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>16</v>
-      </c>
-      <c r="B10">
-        <v>10.87</v>
-      </c>
-      <c r="C10">
-        <v>4097</v>
-      </c>
-      <c r="D10">
-        <v>5770</v>
-      </c>
-      <c r="E10">
-        <v>6.35</v>
-      </c>
-      <c r="F10" t="s">
-        <v>17</v>
+        <v>8</v>
+      </c>
+      <c r="B10" s="1">
+        <v>12.15646632996633</v>
+      </c>
+      <c r="C10" s="1">
+        <v>4581.8806397306398</v>
+      </c>
+      <c r="D10" s="1">
+        <v>6452.880471380472</v>
+      </c>
+      <c r="E10" s="1">
+        <v>7.101523569023569</v>
+      </c>
+      <c r="F10" s="1">
+        <v>60.390909090909098</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B11">
-        <v>4.03</v>
-      </c>
-      <c r="C11">
-        <v>1921</v>
-      </c>
-      <c r="D11">
-        <v>1921</v>
-      </c>
-      <c r="E11">
-        <v>6.12</v>
-      </c>
-      <c r="F11" t="s">
-        <v>19</v>
+        <v>9</v>
+      </c>
+      <c r="B11" s="1">
+        <v>4.5069511784511791</v>
+      </c>
+      <c r="C11" s="1">
+        <v>2148.3506734006737</v>
+      </c>
+      <c r="D11" s="1">
+        <v>2148.3506734006737</v>
+      </c>
+      <c r="E11" s="1">
+        <v>6.8443030303030312</v>
+      </c>
+      <c r="F11" s="1">
+        <v>64.953777777777773</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{fd60f3b8-f236-4830-aecc-da0a7fc54679}" enabled="1" method="Standard" siteId="{76f33c20-5979-4408-adf7-8b3c4be95e52}" contentBits="0" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>